<commit_message>
Added new Tc in Sa
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="141" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68C672BB-EAAD-40A1-8504-DCF9ADA374EC}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11C045D8-73CC-4B26-98DD-77D16CF2BFE6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="496">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1526,6 +1526,15 @@
   </si>
   <si>
     <t>Portland41886</t>
+  </si>
+  <si>
+    <t>Satellite location Status Dropdown</t>
+  </si>
+  <si>
+    <t>TC_075</t>
+  </si>
+  <si>
+    <t>hfrbui</t>
   </si>
 </sst>
 </file>
@@ -1549,7 +1558,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1559,12 +1568,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1582,7 +1585,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -1601,9 +1604,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4022,7 +4022,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
@@ -4394,7 +4394,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>483</v>
       </c>
@@ -4420,7 +4420,22 @@
         <v>492</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>495</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="#$%@$%" xr:uid="{5A227241-ECE1-4878-A7FE-E1EBF1CFB34A}"/>

</xml_diff>

<commit_message>
Added new Tc in Satellite location till 118
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11C045D8-73CC-4B26-98DD-77D16CF2BFE6}"/>
+  <xr:revisionPtr revIDLastSave="265" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97CDFE5E-1BDD-4EDE-A545-874355ACB66E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="551">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1535,6 +1535,171 @@
   </si>
   <si>
     <t>hfrbui</t>
+  </si>
+  <si>
+    <t>RegistrationNumber 1 Text field</t>
+  </si>
+  <si>
+    <t>TC_78to 80</t>
+  </si>
+  <si>
+    <t>SDFGH</t>
+  </si>
+  <si>
+    <t>34567</t>
+  </si>
+  <si>
+    <t>$^&amp;*</t>
+  </si>
+  <si>
+    <t>Tc_82 to 84</t>
+  </si>
+  <si>
+    <t>ftybu</t>
+  </si>
+  <si>
+    <t>8561</t>
+  </si>
+  <si>
+    <t>$%^*</t>
+  </si>
+  <si>
+    <t>EPA ID number text field</t>
+  </si>
+  <si>
+    <t>RTGHyhhh</t>
+  </si>
+  <si>
+    <t>852684</t>
+  </si>
+  <si>
+    <t>#$%^</t>
+  </si>
+  <si>
+    <t>TC_86to 88</t>
+  </si>
+  <si>
+    <t>Dot number field</t>
+  </si>
+  <si>
+    <t>tc_89TO91</t>
+  </si>
+  <si>
+    <t>JHGFV</t>
+  </si>
+  <si>
+    <t>865</t>
+  </si>
+  <si>
+    <t>EIN number</t>
+  </si>
+  <si>
+    <t>TC_92to94</t>
+  </si>
+  <si>
+    <t>GFhjjk</t>
+  </si>
+  <si>
+    <t>$%^&amp;*</t>
+  </si>
+  <si>
+    <t>Entity Id number</t>
+  </si>
+  <si>
+    <t>TC_095to97</t>
+  </si>
+  <si>
+    <t>Hjbj</t>
+  </si>
+  <si>
+    <t>45678</t>
+  </si>
+  <si>
+    <t>856369</t>
+  </si>
+  <si>
+    <t>SoS Numbers</t>
+  </si>
+  <si>
+    <t>TC_98to100</t>
+  </si>
+  <si>
+    <t>tfvV</t>
+  </si>
+  <si>
+    <t>3456</t>
+  </si>
+  <si>
+    <t>SIC code</t>
+  </si>
+  <si>
+    <t>TGfghj</t>
+  </si>
+  <si>
+    <t>5896</t>
+  </si>
+  <si>
+    <t>NAICS code</t>
+  </si>
+  <si>
+    <t>guib</t>
+  </si>
+  <si>
+    <t>7556</t>
+  </si>
+  <si>
+    <t>#$%^&amp;*</t>
+  </si>
+  <si>
+    <t>CAGE code</t>
+  </si>
+  <si>
+    <t>TC_101to103</t>
+  </si>
+  <si>
+    <t>TC_104to106</t>
+  </si>
+  <si>
+    <t>T107to 109</t>
+  </si>
+  <si>
+    <t>YGJ</t>
+  </si>
+  <si>
+    <t>$%^</t>
+  </si>
+  <si>
+    <t>Name text field</t>
+  </si>
+  <si>
+    <t>TC_110to112</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>84658</t>
+  </si>
+  <si>
+    <t>TC_114to116</t>
+  </si>
+  <si>
+    <t>KJN</t>
+  </si>
+  <si>
+    <t>3356</t>
+  </si>
+  <si>
+    <t>(*&amp;%^</t>
+  </si>
+  <si>
+    <t>Street text field</t>
+  </si>
+  <si>
+    <t>Valid Street Address</t>
+  </si>
+  <si>
+    <t>1237 3rd Street Southeast</t>
   </si>
 </sst>
 </file>
@@ -4022,14 +4187,14 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
     <col min="2" max="2" width="25" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="6"/>
     <col min="4" max="4" width="20.77734375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" style="6" customWidth="1"/>
     <col min="6" max="6" width="20.6640625" style="6" customWidth="1"/>
     <col min="7" max="7" width="18.88671875" style="6" customWidth="1"/>
     <col min="8" max="8" width="13.109375" style="6" bestFit="1" customWidth="1"/>
@@ -4434,6 +4599,348 @@
       </c>
       <c r="B39" s="6" t="s">
         <v>495</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>503</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>507</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>529</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A62" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>550</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new Tc in Satellite Loc
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97CDFE5E-1BDD-4EDE-A545-874355ACB66E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{23961DE5-6854-4D5A-8159-BCE975D26128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,6 +20,7 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1699,7 +1695,7 @@
     <t>Valid Street Address</t>
   </si>
   <si>
-    <t>1237 3rd Street Southeast</t>
+    <t>1237 3rd Street</t>
   </si>
 </sst>
 </file>
@@ -1787,10 +1783,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4926,7 +4918,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
         <v>544</v>
       </c>

</xml_diff>

<commit_message>
Added New TC in SAtellite location
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{23961DE5-6854-4D5A-8159-BCE975D26128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="302" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC61DF14-B5D8-4263-B1A0-A677B7EFAA31}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +25,6 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="570">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1696,6 +1700,63 @@
   </si>
   <si>
     <t>1237 3rd Street</t>
+  </si>
+  <si>
+    <t>Suite Text field</t>
+  </si>
+  <si>
+    <t>TC_120to122</t>
+  </si>
+  <si>
+    <t>huenf</t>
+  </si>
+  <si>
+    <t>56464</t>
+  </si>
+  <si>
+    <t>%*($%^**</t>
+  </si>
+  <si>
+    <t>City text field</t>
+  </si>
+  <si>
+    <t>Special Char</t>
+  </si>
+  <si>
+    <t>TC_124to126</t>
+  </si>
+  <si>
+    <t>lnege</t>
+  </si>
+  <si>
+    <t>987</t>
+  </si>
+  <si>
+    <t>^%$#</t>
+  </si>
+  <si>
+    <t>State Txet field</t>
+  </si>
+  <si>
+    <t>TC_129 to 131</t>
+  </si>
+  <si>
+    <t>Fcjbk</t>
+  </si>
+  <si>
+    <t>84889</t>
+  </si>
+  <si>
+    <t>Zip code text field</t>
+  </si>
+  <si>
+    <t>TC_133 to135</t>
+  </si>
+  <si>
+    <t>Iuhnjn</t>
+  </si>
+  <si>
+    <t>2616</t>
   </si>
 </sst>
 </file>
@@ -1783,6 +1844,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4179,7 +4244,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
@@ -4933,6 +4998,118 @@
       </c>
       <c r="E63" s="6" t="s">
         <v>550</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>554</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>569</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added New Tc in Satellite Location Till TC_177
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="302" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC61DF14-B5D8-4263-B1A0-A677B7EFAA31}"/>
+  <xr:revisionPtr revIDLastSave="397" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{207CCBAC-E743-4CE0-8DFE-017C4B410FC9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="615">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1757,6 +1757,141 @@
   </si>
   <si>
     <t>2616</t>
+  </si>
+  <si>
+    <t>Email Text field</t>
+  </si>
+  <si>
+    <t>TC_137to140</t>
+  </si>
+  <si>
+    <t>balli123@gmail.com</t>
+  </si>
+  <si>
+    <t>HUIhfur</t>
+  </si>
+  <si>
+    <t>43143</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid </t>
+  </si>
+  <si>
+    <t>com.@@.com</t>
+  </si>
+  <si>
+    <t>Valid mail ID</t>
+  </si>
+  <si>
+    <t>ballu123@gmail.com</t>
+  </si>
+  <si>
+    <t>Phone number Text field</t>
+  </si>
+  <si>
+    <t>TC_144 to 147</t>
+  </si>
+  <si>
+    <t>243643</t>
+  </si>
+  <si>
+    <t>hbhjbef</t>
+  </si>
+  <si>
+    <t>5646548488</t>
+  </si>
+  <si>
+    <t>$%^&amp;*(</t>
+  </si>
+  <si>
+    <t>Ext text field</t>
+  </si>
+  <si>
+    <t>Tc_149 to 152</t>
+  </si>
+  <si>
+    <t>58975</t>
+  </si>
+  <si>
+    <t>ugi</t>
+  </si>
+  <si>
+    <t>85988</t>
+  </si>
+  <si>
+    <t>&amp;^%@</t>
+  </si>
+  <si>
+    <t>More than 5 digits</t>
+  </si>
+  <si>
+    <t>134525</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Satellite Billing Information</t>
+  </si>
+  <si>
+    <t>Tc_155to 157</t>
+  </si>
+  <si>
+    <t>veggg</t>
+  </si>
+  <si>
+    <t>64864</t>
+  </si>
+  <si>
+    <t>(*^*%</t>
+  </si>
+  <si>
+    <t>Tc_159to161</t>
+  </si>
+  <si>
+    <t>urig</t>
+  </si>
+  <si>
+    <t>564894</t>
+  </si>
+  <si>
+    <t>*&amp;%#@*</t>
+  </si>
+  <si>
+    <t>TC_165 to167</t>
+  </si>
+  <si>
+    <t>bufrei</t>
+  </si>
+  <si>
+    <t>56156</t>
+  </si>
+  <si>
+    <t>%*%$%</t>
+  </si>
+  <si>
+    <t>TC169to171</t>
+  </si>
+  <si>
+    <t>cdgi</t>
+  </si>
+  <si>
+    <t>64861</t>
+  </si>
+  <si>
+    <t>%*^%^$</t>
+  </si>
+  <si>
+    <t>jhcwvdjc</t>
+  </si>
+  <si>
+    <t>684863</t>
+  </si>
+  <si>
+    <t>(&amp;(*&amp;^%</t>
+  </si>
+  <si>
+    <t>Tc_173 to 175</t>
   </si>
 </sst>
 </file>
@@ -1780,7 +1915,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1790,6 +1925,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1807,7 +1948,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -1826,6 +1967,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4244,7 +4388,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
@@ -5014,7 +5158,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>552</v>
       </c>
@@ -5028,7 +5172,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="66" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>556</v>
       </c>
@@ -5042,7 +5186,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>558</v>
       </c>
@@ -5056,7 +5200,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="68" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>562</v>
       </c>
@@ -5070,7 +5214,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>563</v>
       </c>
@@ -5084,7 +5228,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="70" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>566</v>
       </c>
@@ -5098,7 +5242,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>567</v>
       </c>
@@ -5110,6 +5254,277 @@
       </c>
       <c r="D71" s="6" t="s">
         <v>486</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A72" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>572</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A74" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>583</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>590</v>
+      </c>
+      <c r="F77" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" s="10" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>597</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>601</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>612</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>613</v>
       </c>
     </row>
   </sheetData>
@@ -5122,6 +5537,11 @@
     <hyperlink ref="B36" r:id="rId6" xr:uid="{F80053D1-6192-46D4-8135-3162E9DCDBFF}"/>
     <hyperlink ref="F36" r:id="rId7" xr:uid="{A2E87AD7-519E-4D64-A8B0-804F45B567E3}"/>
     <hyperlink ref="G36" r:id="rId8" xr:uid="{001C606C-950A-42AD-84B8-A6A9B9513EE9}"/>
+    <hyperlink ref="B73" r:id="rId9" xr:uid="{24CFF544-36E4-4F50-A277-C01ABB4FEEC2}"/>
+    <hyperlink ref="F73" r:id="rId10" display="com@" xr:uid="{C8CFEF57-B152-49C3-AFFA-70B8D30BAEEE}"/>
+    <hyperlink ref="G73" r:id="rId11" xr:uid="{ACEECA67-88F7-427D-BFAF-783DE7661C96}"/>
+    <hyperlink ref="E77" r:id="rId12" xr:uid="{4E986B8C-EDF0-45DA-B387-2BAFD2E8026F}"/>
+    <hyperlink ref="D82" r:id="rId13" xr:uid="{CDD6978D-1DF9-47A7-99E0-AA10BDC906A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added New Tc Till 199
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="397" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{207CCBAC-E743-4CE0-8DFE-017C4B410FC9}"/>
+  <xr:revisionPtr revIDLastSave="453" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D75C365-79A9-4651-A1C8-33FF86795767}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="637">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1892,6 +1892,72 @@
   </si>
   <si>
     <t>Tc_173 to 175</t>
+  </si>
+  <si>
+    <t>TC_177 to 179</t>
+  </si>
+  <si>
+    <t>kjhrwiug</t>
+  </si>
+  <si>
+    <t>86969</t>
+  </si>
+  <si>
+    <t>#$%^*(</t>
+  </si>
+  <si>
+    <t>Valid Input</t>
+  </si>
+  <si>
+    <t>TC_181 to 184</t>
+  </si>
+  <si>
+    <t>charlie123@gmail.com</t>
+  </si>
+  <si>
+    <t>GYJgj</t>
+  </si>
+  <si>
+    <t>547831</t>
+  </si>
+  <si>
+    <t>&amp;*%8758</t>
+  </si>
+  <si>
+    <t>TC_188 to 191</t>
+  </si>
+  <si>
+    <t>5897458962</t>
+  </si>
+  <si>
+    <t>jjkwbv</t>
+  </si>
+  <si>
+    <t>1234568759</t>
+  </si>
+  <si>
+    <t>*%8758</t>
+  </si>
+  <si>
+    <t>invalid format</t>
+  </si>
+  <si>
+    <t>Tc_194 to 199</t>
+  </si>
+  <si>
+    <t>58945</t>
+  </si>
+  <si>
+    <t>fedsvs</t>
+  </si>
+  <si>
+    <t>68454</t>
+  </si>
+  <si>
+    <t>^$&amp;*&amp;</t>
+  </si>
+  <si>
+    <t>589745</t>
   </si>
 </sst>
 </file>
@@ -4388,7 +4454,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
@@ -4397,7 +4463,7 @@
     <col min="4" max="4" width="20.77734375" style="6" customWidth="1"/>
     <col min="5" max="5" width="23.5546875" style="6" customWidth="1"/>
     <col min="6" max="6" width="20.6640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="18.88671875" style="6" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="6" customWidth="1"/>
     <col min="8" max="8" width="13.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="8.88671875" style="6"/>
   </cols>
@@ -5415,7 +5481,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="81" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>548</v>
       </c>
@@ -5429,7 +5495,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>599</v>
       </c>
@@ -5443,7 +5509,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="83" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>551</v>
       </c>
@@ -5457,7 +5523,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>603</v>
       </c>
@@ -5471,7 +5537,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="85" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>556</v>
       </c>
@@ -5485,7 +5551,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>607</v>
       </c>
@@ -5499,7 +5565,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="87" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>562</v>
       </c>
@@ -5513,7 +5579,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>614</v>
       </c>
@@ -5525,6 +5591,160 @@
       </c>
       <c r="D88" s="6" t="s">
         <v>613</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A91" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="B92" s="9" t="s">
+        <v>621</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="G92" s="9" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A93" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>626</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>628</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A95" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>632</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="D96" s="8" t="s">
+        <v>634</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>636</v>
+      </c>
+      <c r="G96" s="8" t="s">
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -5542,6 +5762,8 @@
     <hyperlink ref="G73" r:id="rId11" xr:uid="{ACEECA67-88F7-427D-BFAF-783DE7661C96}"/>
     <hyperlink ref="E77" r:id="rId12" xr:uid="{4E986B8C-EDF0-45DA-B387-2BAFD2E8026F}"/>
     <hyperlink ref="D82" r:id="rId13" xr:uid="{CDD6978D-1DF9-47A7-99E0-AA10BDC906A5}"/>
+    <hyperlink ref="B92" r:id="rId14" xr:uid="{15FDAB5F-0AF4-4F79-8B5D-CA436D3B9DC1}"/>
+    <hyperlink ref="G92" r:id="rId15" xr:uid="{224A48AA-0076-41B6-B0C3-F943D56C406C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new Tc till 236 in Satellite locations
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="453" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D75C365-79A9-4651-A1C8-33FF86795767}"/>
+  <xr:revisionPtr revIDLastSave="530" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{487847B1-0404-48C1-AF40-949DD44A65EA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="673">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1958,6 +1958,114 @@
   </si>
   <si>
     <t>589745</t>
+  </si>
+  <si>
+    <t>Valid name</t>
+  </si>
+  <si>
+    <t>Naren</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>90210</t>
+  </si>
+  <si>
+    <t>Exact Phone Number</t>
+  </si>
+  <si>
+    <t>8596478598</t>
+  </si>
+  <si>
+    <t>Dispatch Department</t>
+  </si>
+  <si>
+    <t>invalid input</t>
+  </si>
+  <si>
+    <t>TC_211 to215</t>
+  </si>
+  <si>
+    <t>jcwdc</t>
+  </si>
+  <si>
+    <t>657897</t>
+  </si>
+  <si>
+    <t>&amp;%&amp;$%#</t>
+  </si>
+  <si>
+    <t>.com@.com</t>
+  </si>
+  <si>
+    <t>TC_217to220</t>
+  </si>
+  <si>
+    <t>9305948592</t>
+  </si>
+  <si>
+    <t>wufifrwf</t>
+  </si>
+  <si>
+    <t>23434242433</t>
+  </si>
+  <si>
+    <t>*(&amp;(^*&amp;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special char </t>
+  </si>
+  <si>
+    <t>jhqvfew</t>
+  </si>
+  <si>
+    <t>58963</t>
+  </si>
+  <si>
+    <t>%&amp;**%$</t>
+  </si>
+  <si>
+    <t>589632</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>TC_222to228</t>
+  </si>
+  <si>
+    <t>Comapany Display Name</t>
+  </si>
+  <si>
+    <t>Registration number 1</t>
+  </si>
+  <si>
+    <t>General information fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portland </t>
+  </si>
+  <si>
+    <t>5897412563</t>
+  </si>
+  <si>
+    <t>698742</t>
+  </si>
+  <si>
+    <t>Tc_228</t>
+  </si>
+  <si>
+    <t>Dispatch email</t>
+  </si>
+  <si>
+    <t>Dispatch phone</t>
+  </si>
+  <si>
+    <t>naren</t>
+  </si>
+  <si>
+    <t>5896321475</t>
   </si>
 </sst>
 </file>
@@ -4454,12 +4562,12 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
     <col min="2" max="2" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="18.33203125" style="6" customWidth="1"/>
     <col min="4" max="4" width="20.77734375" style="6" customWidth="1"/>
     <col min="5" max="5" width="23.5546875" style="6" customWidth="1"/>
     <col min="6" max="6" width="20.6640625" style="6" customWidth="1"/>
@@ -5161,6 +5269,9 @@
       <c r="D60" s="4" t="s">
         <v>482</v>
       </c>
+      <c r="E60" s="4" t="s">
+        <v>637</v>
+      </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
@@ -5175,6 +5286,9 @@
       <c r="D61" s="6" t="s">
         <v>467</v>
       </c>
+      <c r="E61" s="6" t="s">
+        <v>638</v>
+      </c>
     </row>
     <row r="62" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
@@ -5224,7 +5338,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>552</v>
       </c>
@@ -5238,7 +5352,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>556</v>
       </c>
@@ -5252,7 +5366,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>558</v>
       </c>
@@ -5266,7 +5380,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>562</v>
       </c>
@@ -5280,7 +5394,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>563</v>
       </c>
@@ -5294,7 +5408,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="70" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>566</v>
       </c>
@@ -5307,8 +5421,11 @@
       <c r="D70" s="4" t="s">
         <v>557</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E70" s="4" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>567</v>
       </c>
@@ -5321,8 +5438,11 @@
       <c r="D71" s="6" t="s">
         <v>486</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E71" s="8" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>570</v>
       </c>
@@ -5344,8 +5464,11 @@
       <c r="G72" s="4" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H72" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>571</v>
       </c>
@@ -5367,8 +5490,11 @@
       <c r="G73" s="9" t="s">
         <v>578</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H73" s="6" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>579</v>
       </c>
@@ -5384,8 +5510,11 @@
       <c r="E74" s="4" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F74" s="4" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>580</v>
       </c>
@@ -5401,8 +5530,11 @@
       <c r="E75" s="6" t="s">
         <v>584</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F75" s="8" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>585</v>
       </c>
@@ -5425,7 +5557,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>586</v>
       </c>
@@ -5448,12 +5580,12 @@
         <v>593</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="79" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>540</v>
       </c>
@@ -5467,7 +5599,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>595</v>
       </c>
@@ -5644,7 +5776,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>620</v>
       </c>
@@ -5745,6 +5877,177 @@
       </c>
       <c r="G96" s="8" t="s">
         <v>460</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" s="10" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A98" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>621</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>647</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>649</v>
+      </c>
+      <c r="G99" s="9" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>655</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="D103" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>659</v>
+      </c>
+      <c r="G103" s="8" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A105" s="4" t="s">
+        <v>664</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>666</v>
+      </c>
+      <c r="D106" s="8" t="s">
+        <v>667</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>672</v>
       </c>
     </row>
   </sheetData>
@@ -5764,6 +6067,8 @@
     <hyperlink ref="D82" r:id="rId13" xr:uid="{CDD6978D-1DF9-47A7-99E0-AA10BDC906A5}"/>
     <hyperlink ref="B92" r:id="rId14" xr:uid="{15FDAB5F-0AF4-4F79-8B5D-CA436D3B9DC1}"/>
     <hyperlink ref="G92" r:id="rId15" xr:uid="{224A48AA-0076-41B6-B0C3-F943D56C406C}"/>
+    <hyperlink ref="F99" r:id="rId16" xr:uid="{10706437-A8D3-431D-AB38-0D11EC24B8B2}"/>
+    <hyperlink ref="G99" r:id="rId17" display="charlie123@gmail.com" xr:uid="{BE1272E6-3091-460B-92B3-2F7568D11C99}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Tc after Data removed from Dev environment
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="693" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{185F1A87-A207-41A2-9937-420FC0E99E32}"/>
+  <xr:revisionPtr revIDLastSave="696" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCC3B1E4-CBF4-4EED-A889-0D92CC11CE2B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup365" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="804">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="805">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1527,9 +1527,6 @@
     <t>Satellite loaction Name</t>
   </si>
   <si>
-    <t>Portland41886</t>
-  </si>
-  <si>
     <t>Satellite location Status Dropdown</t>
   </si>
   <si>
@@ -2461,6 +2458,12 @@
   </si>
   <si>
     <t>8965741235</t>
+  </si>
+  <si>
+    <t>Charlie waste Management_106893</t>
+  </si>
+  <si>
+    <t>charlie44636</t>
   </si>
 </sst>
 </file>
@@ -3299,12 +3302,12 @@
         <v>490</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>492</v>
+        <v>804</v>
       </c>
     </row>
     <row r="38" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>475</v>
@@ -3312,15 +3315,15 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>494</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>406</v>
@@ -3334,21 +3337,21 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="B41" s="6" t="s">
         <v>497</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="C41" s="8" t="s">
         <v>498</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="D41" s="6" t="s">
         <v>499</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>406</v>
@@ -3362,21 +3365,21 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="C43" s="8" t="s">
         <v>502</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="D43" s="6" t="s">
         <v>503</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>406</v>
@@ -3390,21 +3393,21 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B45" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>506</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="D45" s="6" t="s">
         <v>507</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>406</v>
@@ -3418,13 +3421,13 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>511</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="C47" s="8" t="s">
         <v>512</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>513</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>486</v>
@@ -3432,7 +3435,7 @@
     </row>
     <row r="48" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>406</v>
@@ -3446,21 +3449,21 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="B49" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="C49" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>516</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>522</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>406</v>
@@ -3474,13 +3477,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>519</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="C51" s="8" t="s">
         <v>520</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>521</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>467</v>
@@ -3488,7 +3491,7 @@
     </row>
     <row r="52" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>406</v>
@@ -3502,21 +3505,21 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>524</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="C53" s="8" t="s">
         <v>525</v>
       </c>
-      <c r="C53" s="8" t="s">
-        <v>526</v>
-      </c>
       <c r="D53" s="6" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>406</v>
@@ -3530,21 +3533,21 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B55" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="C55" s="8" t="s">
         <v>528</v>
       </c>
-      <c r="C55" s="8" t="s">
-        <v>529</v>
-      </c>
       <c r="D55" s="6" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>406</v>
@@ -3558,21 +3561,21 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B57" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="C57" s="8" t="s">
         <v>531</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="D57" s="6" t="s">
         <v>532</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>406</v>
@@ -3586,21 +3589,21 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="B59" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="C59" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>538</v>
-      </c>
-      <c r="C59" s="8" t="s">
-        <v>499</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>406</v>
@@ -3612,29 +3615,29 @@
         <v>482</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="B61" s="6" t="s">
         <v>541</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="C61" s="8" t="s">
         <v>542</v>
-      </c>
-      <c r="C61" s="8" t="s">
-        <v>543</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>467</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>406</v>
@@ -3646,29 +3649,29 @@
         <v>482</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="B63" s="6" t="s">
         <v>544</v>
       </c>
-      <c r="B63" s="6" t="s">
+      <c r="C63" s="8" t="s">
         <v>545</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="D63" s="6" t="s">
         <v>546</v>
       </c>
-      <c r="D63" s="6" t="s">
-        <v>547</v>
-      </c>
       <c r="E63" s="6" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>406</v>
@@ -3682,21 +3685,21 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="B65" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="B65" s="6" t="s">
+      <c r="C65" s="8" t="s">
         <v>553</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="D65" s="6" t="s">
         <v>554</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>406</v>
@@ -3705,26 +3708,26 @@
         <v>388</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="B67" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="B67" s="6" t="s">
+      <c r="C67" s="8" t="s">
         <v>559</v>
       </c>
-      <c r="C67" s="8" t="s">
+      <c r="D67" s="6" t="s">
         <v>560</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="68" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>406</v>
@@ -3733,18 +3736,18 @@
         <v>388</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>563</v>
       </c>
-      <c r="B69" s="6" t="s">
+      <c r="C69" s="8" t="s">
         <v>564</v>
-      </c>
-      <c r="C69" s="8" t="s">
-        <v>565</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>467</v>
@@ -3752,7 +3755,7 @@
     </row>
     <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>406</v>
@@ -3761,32 +3764,32 @@
         <v>388</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="B71" s="6" t="s">
         <v>567</v>
       </c>
-      <c r="B71" s="6" t="s">
+      <c r="C71" s="8" t="s">
         <v>568</v>
-      </c>
-      <c r="C71" s="8" t="s">
-        <v>569</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>486</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="72" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>475</v>
@@ -3801,10 +3804,10 @@
         <v>482</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="H72" s="4" t="s">
         <v>1</v>
@@ -3812,33 +3815,33 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="B73" s="9" t="s">
         <v>571</v>
       </c>
-      <c r="B73" s="9" t="s">
+      <c r="C73" s="6" t="s">
         <v>572</v>
       </c>
-      <c r="C73" s="6" t="s">
+      <c r="D73" s="8" t="s">
         <v>573</v>
       </c>
-      <c r="D73" s="8" t="s">
-        <v>574</v>
-      </c>
       <c r="E73" s="6" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="74" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>475</v>
@@ -3853,32 +3856,32 @@
         <v>398</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B75" s="8" t="s">
         <v>580</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="C75" s="6" t="s">
         <v>581</v>
       </c>
-      <c r="C75" s="6" t="s">
+      <c r="D75" s="8" t="s">
         <v>582</v>
       </c>
-      <c r="D75" s="8" t="s">
+      <c r="E75" s="6" t="s">
         <v>583</v>
       </c>
-      <c r="E75" s="6" t="s">
-        <v>584</v>
-      </c>
       <c r="F75" s="8" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="76" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>475</v>
@@ -3893,7 +3896,7 @@
         <v>398</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>453</v>
@@ -3901,35 +3904,35 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="B77" s="8" t="s">
         <v>586</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="C77" s="6" t="s">
         <v>587</v>
       </c>
-      <c r="C77" s="6" t="s">
+      <c r="D77" s="8" t="s">
         <v>588</v>
       </c>
-      <c r="D77" s="8" t="s">
+      <c r="E77" s="9" t="s">
         <v>589</v>
       </c>
-      <c r="E77" s="9" t="s">
-        <v>590</v>
-      </c>
       <c r="F77" s="8" t="s">
+        <v>591</v>
+      </c>
+      <c r="G77" s="8" t="s">
         <v>592</v>
-      </c>
-      <c r="G77" s="8" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="79" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>406</v>
@@ -3943,21 +3946,21 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="B80" s="6" t="s">
         <v>595</v>
       </c>
-      <c r="B80" s="6" t="s">
+      <c r="C80" s="8" t="s">
         <v>596</v>
       </c>
-      <c r="C80" s="8" t="s">
+      <c r="D80" s="6" t="s">
         <v>597</v>
-      </c>
-      <c r="D80" s="6" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="81" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>406</v>
@@ -3966,26 +3969,26 @@
         <v>388</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="B82" s="6" t="s">
         <v>599</v>
       </c>
-      <c r="B82" s="6" t="s">
+      <c r="C82" s="8" t="s">
         <v>600</v>
       </c>
-      <c r="C82" s="8" t="s">
+      <c r="D82" s="9" t="s">
         <v>601</v>
-      </c>
-      <c r="D82" s="9" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="83" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>406</v>
@@ -3999,21 +4002,21 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="B84" s="6" t="s">
         <v>603</v>
       </c>
-      <c r="B84" s="6" t="s">
+      <c r="C84" s="8" t="s">
         <v>604</v>
       </c>
-      <c r="C84" s="8" t="s">
+      <c r="D84" s="6" t="s">
         <v>605</v>
-      </c>
-      <c r="D84" s="6" t="s">
-        <v>606</v>
       </c>
     </row>
     <row r="85" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>406</v>
@@ -4027,21 +4030,21 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="B86" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="B86" s="6" t="s">
+      <c r="C86" s="8" t="s">
         <v>608</v>
       </c>
-      <c r="C86" s="8" t="s">
+      <c r="D86" s="6" t="s">
         <v>609</v>
-      </c>
-      <c r="D86" s="6" t="s">
-        <v>610</v>
       </c>
     </row>
     <row r="87" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>406</v>
@@ -4050,26 +4053,26 @@
         <v>388</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B88" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="C88" s="8" t="s">
         <v>611</v>
       </c>
-      <c r="C88" s="8" t="s">
+      <c r="D88" s="6" t="s">
         <v>612</v>
-      </c>
-      <c r="D88" s="6" t="s">
-        <v>613</v>
       </c>
     </row>
     <row r="89" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>406</v>
@@ -4083,24 +4086,24 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="B90" s="6" t="s">
         <v>615</v>
       </c>
-      <c r="B90" s="6" t="s">
+      <c r="C90" s="8" t="s">
         <v>616</v>
       </c>
-      <c r="C90" s="8" t="s">
+      <c r="D90" s="6" t="s">
         <v>617</v>
-      </c>
-      <c r="D90" s="6" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="91" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>406</v>
@@ -4112,38 +4115,38 @@
         <v>482</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
+        <v>619</v>
+      </c>
+      <c r="B92" s="9" t="s">
         <v>620</v>
       </c>
-      <c r="B92" s="9" t="s">
+      <c r="C92" s="6" t="s">
         <v>621</v>
       </c>
-      <c r="C92" s="6" t="s">
+      <c r="D92" s="8" t="s">
         <v>622</v>
       </c>
-      <c r="D92" s="8" t="s">
+      <c r="E92" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="E92" s="6" t="s">
-        <v>624</v>
-      </c>
       <c r="F92" s="6" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="93" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>446</v>
@@ -4155,32 +4158,32 @@
         <v>388</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="B94" s="8" t="s">
         <v>625</v>
       </c>
-      <c r="B94" s="8" t="s">
+      <c r="C94" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="C94" s="6" t="s">
+      <c r="D94" s="8" t="s">
         <v>627</v>
       </c>
-      <c r="D94" s="8" t="s">
+      <c r="E94" s="6" t="s">
         <v>628</v>
-      </c>
-      <c r="E94" s="6" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="95" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>406</v>
@@ -4192,7 +4195,7 @@
         <v>398</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G95" s="4" t="s">
         <v>453</v>
@@ -4200,22 +4203,22 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="B96" s="8" t="s">
         <v>631</v>
       </c>
-      <c r="B96" s="8" t="s">
+      <c r="C96" s="6" t="s">
         <v>632</v>
       </c>
-      <c r="C96" s="6" t="s">
+      <c r="D96" s="8" t="s">
         <v>633</v>
       </c>
-      <c r="D96" s="8" t="s">
+      <c r="E96" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="E96" s="6" t="s">
+      <c r="F96" s="8" t="s">
         <v>635</v>
-      </c>
-      <c r="F96" s="8" t="s">
-        <v>636</v>
       </c>
       <c r="G96" s="8" t="s">
         <v>460</v>
@@ -4223,12 +4226,12 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="10" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="98" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>475</v>
@@ -4243,30 +4246,30 @@
         <v>482</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>620</v>
+      </c>
+      <c r="C99" s="6" t="s">
         <v>645</v>
       </c>
-      <c r="B99" s="8" t="s">
-        <v>621</v>
-      </c>
-      <c r="C99" s="6" t="s">
+      <c r="D99" s="8" t="s">
         <v>646</v>
       </c>
-      <c r="D99" s="8" t="s">
+      <c r="E99" s="6" t="s">
         <v>647</v>
       </c>
-      <c r="E99" s="6" t="s">
+      <c r="F99" s="9" t="s">
         <v>648</v>
-      </c>
-      <c r="F99" s="9" t="s">
-        <v>649</v>
       </c>
       <c r="G99" s="9" t="s">
         <v>392</v>
@@ -4274,7 +4277,7 @@
     </row>
     <row r="100" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>475</v>
@@ -4291,24 +4294,24 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="B101" s="8" t="s">
         <v>650</v>
       </c>
-      <c r="B101" s="8" t="s">
+      <c r="C101" s="6" t="s">
         <v>651</v>
       </c>
-      <c r="C101" s="6" t="s">
+      <c r="D101" s="8" t="s">
         <v>652</v>
       </c>
-      <c r="D101" s="8" t="s">
+      <c r="E101" s="6" t="s">
         <v>653</v>
-      </c>
-      <c r="E101" s="6" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="102" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>475</v>
@@ -4320,10 +4323,10 @@
         <v>388</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G102" s="4" t="s">
         <v>453</v>
@@ -4331,65 +4334,65 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C103" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="D103" s="8" t="s">
         <v>656</v>
       </c>
-      <c r="D103" s="8" t="s">
+      <c r="E103" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="E103" s="6" t="s">
+      <c r="F103" s="8" t="s">
         <v>658</v>
       </c>
-      <c r="F103" s="8" t="s">
+      <c r="G103" s="8" t="s">
         <v>659</v>
-      </c>
-      <c r="G103" s="8" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="105" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>445</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E105" s="4" t="s">
+        <v>668</v>
+      </c>
+      <c r="F105" s="4" t="s">
         <v>669</v>
-      </c>
-      <c r="F105" s="4" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B106" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="C106" s="8" t="s">
         <v>665</v>
       </c>
-      <c r="C106" s="8" t="s">
+      <c r="D106" s="8" t="s">
         <v>666</v>
       </c>
-      <c r="D106" s="8" t="s">
-        <v>667</v>
-      </c>
       <c r="E106" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="F106" s="8" t="s">
         <v>671</v>
-      </c>
-      <c r="F106" s="8" t="s">
-        <v>672</v>
       </c>
     </row>
   </sheetData>
@@ -4479,15 +4482,15 @@
         <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>672</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>673</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>321</v>
@@ -4501,18 +4504,18 @@
         <v>15</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>675</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>676</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>677</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>678</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B8" t="s">
         <v>320</v>
@@ -4529,18 +4532,18 @@
         <v>15</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>681</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>682</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B11" t="s">
         <v>320</v>
@@ -4557,18 +4560,18 @@
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>683</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>684</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>685</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B14" t="s">
         <v>320</v>
@@ -4585,27 +4588,27 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>688</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>689</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>690</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>691</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>692</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>693</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>256</v>
@@ -4620,10 +4623,10 @@
         <v>238</v>
       </c>
       <c r="F17" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>695</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -4634,7 +4637,7 @@
         <v>228</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>158</v>
@@ -4643,10 +4646,10 @@
         <v>159</v>
       </c>
       <c r="F19" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="G19" s="3" t="s">
         <v>698</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>699</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -4666,7 +4669,7 @@
         <v>238</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>264</v>
@@ -4677,24 +4680,24 @@
         <v>15</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>700</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>701</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>702</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>703</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>704</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>705</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B23" t="s">
         <v>320</v>
@@ -4706,10 +4709,10 @@
         <v>238</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>707</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -4717,18 +4720,18 @@
         <v>15</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>709</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>710</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>711</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B26" t="s">
         <v>320</v>
@@ -4745,10 +4748,10 @@
         <v>15</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>713</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>714</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>99</v>
@@ -4756,7 +4759,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B29" t="s">
         <v>320</v>
@@ -4784,7 +4787,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B32" t="s">
         <v>320</v>
@@ -4812,7 +4815,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B35" t="s">
         <v>320</v>
@@ -4835,12 +4838,12 @@
         <v>129</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B38" t="s">
         <v>320</v>
@@ -4857,21 +4860,21 @@
         <v>15</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>720</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>721</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>138</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B41" t="s">
         <v>320</v>
@@ -4883,7 +4886,7 @@
         <v>238</v>
       </c>
       <c r="E41" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -4903,12 +4906,12 @@
         <v>253</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B44" t="s">
         <v>320</v>
@@ -4920,10 +4923,10 @@
         <v>238</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>727</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -4943,7 +4946,7 @@
         <v>260</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -4954,16 +4957,16 @@
         <v>320</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D47" t="s">
         <v>238</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>730</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>731</v>
       </c>
     </row>
   </sheetData>
@@ -4977,10 +4980,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77142416-745D-4F9D-B8CB-E786E8AF6BF4}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -5005,6 +5008,11 @@
       </c>
       <c r="D2" t="s">
         <v>416</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>803</v>
       </c>
     </row>
   </sheetData>
@@ -5028,10 +5036,10 @@
   <sheetData>
     <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>406</v>
@@ -5045,27 +5053,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>733</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>734</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="D2" s="13" t="s">
         <v>735</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="11" t="s">
         <v>736</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>406</v>
@@ -5074,64 +5082,64 @@
         <v>388</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>737</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>738</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="13" t="s">
         <v>739</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>740</v>
-      </c>
       <c r="E5" s="11" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>743</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>744</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>475</v>
@@ -5146,58 +5154,58 @@
         <v>482</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
+        <v>750</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>751</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="C14" s="11" t="s">
         <v>752</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="D14" s="13" t="s">
         <v>753</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>754</v>
-      </c>
       <c r="E14" s="11" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
+        <v>756</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>757</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>758</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>406</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
+        <v>759</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>760</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="C16" s="11" t="s">
         <v>761</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="D16" s="13" t="s">
         <v>762</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>763</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>443</v>
@@ -5205,179 +5213,179 @@
     </row>
     <row r="17" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>406</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
+        <v>765</v>
+      </c>
+      <c r="B18" s="11" t="s">
         <v>766</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="C18" s="13" t="s">
         <v>767</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="D18" s="13" t="s">
         <v>768</v>
       </c>
-      <c r="D18" s="13" t="s">
-        <v>769</v>
-      </c>
       <c r="E18" s="11" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>406</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
+        <v>773</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>774</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="C22" s="11" t="s">
         <v>775</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="D22" s="13" t="s">
         <v>776</v>
       </c>
-      <c r="D22" s="13" t="s">
-        <v>777</v>
-      </c>
       <c r="E22" s="11" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="23" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>406</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
+        <v>778</v>
+      </c>
+      <c r="B24" s="13" t="s">
         <v>779</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="C24" s="11" t="s">
         <v>780</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="D24" s="13" t="s">
         <v>781</v>
       </c>
-      <c r="D24" s="13" t="s">
-        <v>782</v>
-      </c>
       <c r="E24" s="11" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>406</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
+        <v>783</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>784</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="C26" s="11" t="s">
         <v>785</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="D26" s="13" t="s">
         <v>786</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="E26" s="14" t="s">
         <v>787</v>
       </c>
-      <c r="E26" s="14" t="s">
-        <v>788</v>
-      </c>
       <c r="F26" s="13" t="s">
+        <v>789</v>
+      </c>
+      <c r="G26" s="13" t="s">
         <v>790</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>476</v>
@@ -5385,7 +5393,7 @@
     </row>
     <row r="29" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>406</v>
@@ -5399,16 +5407,16 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
+        <v>794</v>
+      </c>
+      <c r="B30" s="11" t="s">
         <v>795</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="C30" s="13" t="s">
         <v>796</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>797</v>
-      </c>
       <c r="D30" s="11" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>
@@ -5440,13 +5448,13 @@
         <v>77</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>799</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>800</v>
-      </c>
       <c r="E1" s="3" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -5454,16 +5462,16 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel sheet merged with Nagaveni
</commit_message>
<xml_diff>
--- a/Octopussaas_main_Framework/Test data/read.xlsx
+++ b/Octopussaas_main_Framework/Test data/read.xlsx
@@ -1,23 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="696" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCC3B1E4-CBF4-4EED-A889-0D92CC11CE2B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{2AC28ABD-5620-4052-9C7E-703FCFC9F1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup365" sheetId="1" r:id="rId1"/>
     <sheet name="Generator" sheetId="10" r:id="rId2"/>
-    <sheet name="Disposal Facillity" sheetId="11" r:id="rId3"/>
-    <sheet name="Unapplied checks" sheetId="12" r:id="rId4"/>
-    <sheet name="Routeassignment" sheetId="3" r:id="rId5"/>
+    <sheet name="Routeassignment" sheetId="3" r:id="rId3"/>
+    <sheet name="Disposal Facillity" sheetId="11" r:id="rId4"/>
+    <sheet name="Unapplied checks" sheetId="12" r:id="rId5"/>
     <sheet name="TransporterProfile" sheetId="2" r:id="rId6"/>
     <sheet name="MyProfile" sheetId="4" r:id="rId7"/>
     <sheet name="Drivers" sheetId="5" r:id="rId8"/>
@@ -27,6 +22,7 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A15:N25"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2572,10 +2568,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3635,7 +3627,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>547</v>
       </c>
@@ -3787,7 +3779,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>569</v>
       </c>
@@ -3839,7 +3831,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="74" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>578</v>
       </c>
@@ -3879,7 +3871,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="76" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>584</v>
       </c>
@@ -4098,7 +4090,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="91" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>569</v>
       </c>
@@ -4144,7 +4136,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="93" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>578</v>
       </c>
@@ -4178,7 +4170,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="95" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>584</v>
       </c>
@@ -4229,7 +4221,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="98" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>569</v>
       </c>
@@ -4275,7 +4267,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="100" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>578</v>
       </c>
@@ -4309,7 +4301,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="102" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>584</v>
       </c>
@@ -5021,6 +5013,152 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C6CDDE-28EE-4E4D-95AF-5786FC71BBC0}">
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" t="s">
+        <v>423</v>
+      </c>
+      <c r="C5" t="s">
+        <v>424</v>
+      </c>
+      <c r="D5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E5" t="s">
+        <v>426</v>
+      </c>
+      <c r="F5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>428</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B11" t="s">
+        <v>432</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{96BF7A5F-3686-41FE-B674-C9DCD2DB7544}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB07B270-85DC-4F6D-8AC7-D93CAE493508}">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5429,7 +5567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16196D24-437F-4113-984C-E1E07E6FEFBB}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5477,152 +5615,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{FA134B35-6A03-43B7-BC3C-F6C686D80E46}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C6CDDE-28EE-4E4D-95AF-5786FC71BBC0}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>422</v>
-      </c>
-      <c r="B5" t="s">
-        <v>423</v>
-      </c>
-      <c r="C5" t="s">
-        <v>424</v>
-      </c>
-      <c r="D5" t="s">
-        <v>425</v>
-      </c>
-      <c r="E5" t="s">
-        <v>426</v>
-      </c>
-      <c r="F5" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>427</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-    </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>428</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>431</v>
-      </c>
-      <c r="B11" t="s">
-        <v>432</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{96BF7A5F-3686-41FE-B674-C9DCD2DB7544}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>